<commit_message>
chore: update daily stock screen report
</commit_message>
<xml_diff>
--- a/reports/holding_plan.xlsx
+++ b/reports/holding_plan.xlsx
@@ -98,7 +98,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -311,7 +311,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -398,7 +398,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-13 20:17:51</t>
+          <t>2026-06-14 19:15:44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1276,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="6" max="6" width="60" customWidth="1"/>
@@ -1335,6 +1335,32 @@
         <v>3</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>aiHF skipped: missing LLM API key secret</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-14 19:15:44</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>aiHF skipped: missing LLM API key secret</t>
         </is>

</xml_diff>